<commit_message>
populate QADive sheet with remaining tests
</commit_message>
<xml_diff>
--- a/Excel file summary.xlsx
+++ b/Excel file summary.xlsx
@@ -5,26 +5,27 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unigeit-my.sharepoint.com/personal/s3925210_studenti_unige_it/Documents/MSc/FSTT/Functional/project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mezaj\projects\fstt_assignment\maven_selenium_project_Petclinic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{EDAF49EA-6D5B-42AC-983B-4E106A0D9A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8696D29C-0172-4EE6-967F-02A00CD5FD19}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BA5C2E-577E-4F7C-A7F1-4E0CFA97E343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="615" windowWidth="19395" windowHeight="20355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="615" windowWidth="38580" windowHeight="20355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Results" sheetId="1" r:id="rId1"/>
-    <sheet name="Classification Guide" sheetId="2" r:id="rId2"/>
+    <sheet name="QADive" sheetId="1" r:id="rId1"/>
+    <sheet name="Results" sheetId="2" r:id="rId2"/>
+    <sheet name="Classification Guide" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Results!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Results!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="94">
   <si>
     <t>App</t>
   </si>
@@ -62,6 +63,129 @@
     <t>Manual Notes</t>
   </si>
   <si>
+    <t>PetClinic</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyAddress</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyAdressM</t>
+  </si>
+  <si>
+    <t>Without comments</t>
+  </si>
+  <si>
+    <t>Gemma 4-31B-IT</t>
+  </si>
+  <si>
+    <t>With comments</t>
+  </si>
+  <si>
+    <t>With comments plus web pages</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyCity</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyCityM</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyFirstName</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyFirstNameM</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyLastName</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyLastNameM</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyTelephone</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithEmptyTelephoneM</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithLongTelephone</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithLongTelephoneM</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithNotNumericTelephone</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithNotNumericTelephoneM</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithValidData</t>
+  </si>
+  <si>
+    <t>TestAddOwnerWithValidDataM</t>
+  </si>
+  <si>
+    <t>TestEditOwnerEmptyField</t>
+  </si>
+  <si>
+    <t>TestEditOwnerEmptyFieldM</t>
+  </si>
+  <si>
+    <t>TestEditOwnerWithLongTelephone</t>
+  </si>
+  <si>
+    <t>TestEditOwnerWithLongTelephoneM</t>
+  </si>
+  <si>
+    <t>TestEditOwnerWithNotNumericTelephone</t>
+  </si>
+  <si>
+    <t>TestEditOwnerWithNotNumericTelephoneM</t>
+  </si>
+  <si>
+    <t>TestEditOwnerWithValidData</t>
+  </si>
+  <si>
+    <t>TestEditOwnerWithValidDataM</t>
+  </si>
+  <si>
+    <t>TestFindAllOwner</t>
+  </si>
+  <si>
+    <t>TestFindAllOwnerM</t>
+  </si>
+  <si>
+    <t>TestFindExistingOwner</t>
+  </si>
+  <si>
+    <t>TestFindExistingOwnerM</t>
+  </si>
+  <si>
+    <t>TestFindExistingOwnerFromAll</t>
+  </si>
+  <si>
+    <t>TestFindExistingOwnerFromAllM</t>
+  </si>
+  <si>
+    <t>TestFindNotExistingOwner</t>
+  </si>
+  <si>
+    <t>TestFindNotExistingOwnerM</t>
+  </si>
+  <si>
+    <t>TestPetToOwner</t>
+  </si>
+  <si>
+    <t>TestPetToOwnerM</t>
+  </si>
+  <si>
+    <t>TestPetToOwnerWithEmptyField</t>
+  </si>
+  <si>
+    <t>TestPetToOwnerWithEmptyFieldM</t>
+  </si>
+  <si>
     <t>mantisbt</t>
   </si>
   <si>
@@ -71,7 +195,16 @@
     <t>addCategory</t>
   </si>
   <si>
+    <t>Gemma-4-31B-it</t>
+  </si>
+  <si>
     <t>assertEquals(categoryName, editProj.getProjectCategory());</t>
+  </si>
+  <si>
+    <t>assertEquals(categoryName, editProj.getCategory());</t>
+  </si>
+  <si>
+    <t>RUN TIME ERROR</t>
   </si>
   <si>
     <t>no such element: Unable to locate element: {"method":"xpath","selector":"//*[@id="categories"]/div/div[3]/div/div/table/tbody/tr[1]/td[1]"}
@@ -82,21 +215,24 @@
 Driver info: org.open</t>
   </si>
   <si>
+    <t>wrong_assertion</t>
+  </si>
+  <si>
+    <t>AddEmptyUserFailsTest</t>
+  </si>
+  <si>
+    <t>addEmptyUserFails</t>
+  </si>
+  <si>
+    <t>assertEquals(Strings.errorInvalidUser, userPage.getError());</t>
+  </si>
+  <si>
+    <t>PASSED</t>
+  </si>
+  <si>
     <t>correct</t>
   </si>
   <si>
-    <t>AddEmptyUserFailsTest</t>
-  </si>
-  <si>
-    <t>addEmptyUserFails</t>
-  </si>
-  <si>
-    <t>assertEquals(Strings.errorInvalidUser, userPage.getError());</t>
-  </si>
-  <si>
-    <t>wrong_assertion</t>
-  </si>
-  <si>
     <t>assertEquals(userPage.getError(), Strings.errorInvalidUser);</t>
   </si>
   <si>
@@ -127,10 +263,10 @@
     <t>assertEquals("Expected error message not displayed", "Project already exists", project.getError());</t>
   </si>
   <si>
+    <t>FAILED</t>
+  </si>
+  <si>
     <t>Expected error message not displayed expected:&lt;[Project already exists]&gt; but was:&lt;[A project with that name already exists. Please go back and enter a different name.]&gt;</t>
-  </si>
-  <si>
-    <t>not_executable</t>
   </si>
   <si>
     <t>Classification</t>
@@ -173,34 +309,13 @@
 Generated: assertEquals("admin", page.getAccessLevel(1))</t>
   </si>
   <si>
+    <t>not_executable</t>
+  </si>
+  <si>
     <t>Does not compile or cannot run</t>
   </si>
   <si>
     <t>Syntax error, missing method, wrong locator</t>
-  </si>
-  <si>
-    <t>Without comments</t>
-  </si>
-  <si>
-    <t>With comments</t>
-  </si>
-  <si>
-    <t>With comments plus web pages</t>
-  </si>
-  <si>
-    <t>Gemma-4-31B-it</t>
-  </si>
-  <si>
-    <t>RUN TIME ERROR</t>
-  </si>
-  <si>
-    <t>assertEquals(categoryName, editProj.getCategory());</t>
-  </si>
-  <si>
-    <t>PASSED</t>
-  </si>
-  <si>
-    <t>FAILED</t>
   </si>
 </sst>
 </file>
@@ -255,7 +370,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -289,11 +404,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -317,11 +450,590 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="29">
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center"/>
+      <border outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border outline="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2F5496"/>
+          <bgColor rgb="FF2F5496"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -332,6 +1044,27 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L6" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25" totalsRowBorderDxfId="24">
+  <autoFilter ref="A1:L6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="App" totalsRowLabel="Total" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Class" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Method" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Treatment" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Model" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Gold Standard Assertion" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Generated Assertion" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Compiles" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Pass/Fail" dataDxfId="7" totalsRowDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Fail Reason" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Manual Classification" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Manual Notes" totalsRowFunction="count" dataDxfId="1" totalsRowDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -617,30 +1350,1374 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="42.85546875" customWidth="1"/>
+    <col min="3" max="3" width="34.85546875" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+    </row>
+    <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+    </row>
+    <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+    </row>
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+    </row>
+    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+    </row>
+    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+    </row>
+    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+    </row>
+    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+    </row>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+    </row>
+    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+    </row>
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+    </row>
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+    </row>
+    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+    </row>
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+    </row>
+    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+    </row>
+    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+    </row>
+    <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+    </row>
+    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+    </row>
+    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+    </row>
+    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+    </row>
+    <row r="22" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+    </row>
+    <row r="23" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+    </row>
+    <row r="24" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+    </row>
+    <row r="25" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="12"/>
+    </row>
+    <row r="29" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+    </row>
+    <row r="30" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+    </row>
+    <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+    </row>
+    <row r="32" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+    </row>
+    <row r="33" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="12"/>
+    </row>
+    <row r="34" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+    </row>
+    <row r="35" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="12"/>
+    </row>
+    <row r="36" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="12"/>
+      <c r="L36" s="12"/>
+    </row>
+    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="12"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="12"/>
+      <c r="L38" s="12"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="12"/>
+      <c r="K39" s="12"/>
+      <c r="L39" s="12"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E40" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="12"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E41" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="12"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E43" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="12"/>
+      <c r="L43" s="12"/>
+    </row>
+    <row r="44" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E44" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="12"/>
+      <c r="L44" s="12"/>
+    </row>
+    <row r="45" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="15"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="12"/>
+    </row>
+    <row r="46" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E46" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" s="12"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
+      <c r="L46" s="12"/>
+    </row>
+    <row r="47" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" s="12"/>
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
+      <c r="L47" s="12"/>
+    </row>
+    <row r="48" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F48" s="12"/>
+      <c r="G48" s="12"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="12"/>
+      <c r="K48" s="12"/>
+      <c r="L48" s="12"/>
+    </row>
+    <row r="49" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="15"/>
+      <c r="J49" s="12"/>
+      <c r="K49" s="12"/>
+      <c r="L49" s="12"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F50" s="12"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="12"/>
+      <c r="I50" s="15"/>
+      <c r="J50" s="12"/>
+      <c r="K50" s="12"/>
+      <c r="L50" s="12"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F51" s="12"/>
+      <c r="G51" s="12"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="12"/>
+      <c r="K51" s="12"/>
+      <c r="L51" s="12"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F52" s="12"/>
+      <c r="G52" s="12"/>
+      <c r="H52" s="12"/>
+      <c r="I52" s="15"/>
+      <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="12"/>
+    </row>
+    <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B53" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F53" s="12"/>
+      <c r="G53" s="12"/>
+      <c r="H53" s="12"/>
+      <c r="I53" s="15"/>
+      <c r="J53" s="12"/>
+      <c r="K53" s="12"/>
+      <c r="L53" s="12"/>
+    </row>
+    <row r="54" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" s="12"/>
+      <c r="G54" s="12"/>
+      <c r="H54" s="12"/>
+      <c r="I54" s="15"/>
+      <c r="J54" s="12"/>
+      <c r="K54" s="12"/>
+      <c r="L54" s="12"/>
+    </row>
+    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F55" s="12"/>
+      <c r="G55" s="12"/>
+      <c r="H55" s="12"/>
+      <c r="I55" s="15"/>
+      <c r="J55" s="12"/>
+      <c r="K55" s="12"/>
+      <c r="L55" s="12"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid classification" error="Please select a valid classification" promptTitle="Manual Classification" prompt="Select classification" sqref="K2:K6" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"correct,over_assertive,under_assertive,wrong_assertion,not_executable"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
 
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{E0380448-3BC6-4DEC-A576-2075B45D98A7}">
-  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;28d48dfc-78d4-43bd-9104-f0dcd85ba81c&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -694,245 +2771,245 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="255" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="H2" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="H3" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="E4" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="H4" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="E5" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="H5" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="H6" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
       <c r="H8" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="L8" s="2"/>
     </row>
@@ -940,9 +3017,9 @@
       <c r="D9" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L8" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L8" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid classification" error="Please select a valid classification" promptTitle="Manual Classification" prompt="Select classification" sqref="K2:K8" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid classification" error="Please select a valid classification" promptTitle="Manual Classification" prompt="Select classification" sqref="K2:K8" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"correct,over_assertive,under_assertive,wrong_assertion,not_executable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -950,8 +3027,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -962,68 +3039,68 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
record manual classifications in summary sheet
</commit_message>
<xml_diff>
--- a/Excel file summary.xlsx
+++ b/Excel file summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mezaj\projects\fstt_assignment\maven_selenium_project_Petclinic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BA5C2E-577E-4F7C-A7F1-4E0CFA97E343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF97F064-0C6B-4497-946B-C64C51C47F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="615" windowWidth="38580" windowHeight="20355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19110" yWindow="615" windowWidth="19395" windowHeight="20355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QADive" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="123">
   <si>
     <t>App</t>
   </si>
@@ -78,6 +78,9 @@
     <t>Gemma 4-31B-IT</t>
   </si>
   <si>
+    <t>assertEquals("must not be blank", driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[3]/div[1]/span[2]")) .getText());</t>
+  </si>
+  <si>
     <t>With comments</t>
   </si>
   <si>
@@ -90,30 +93,45 @@
     <t>TestAddOwnerWithEmptyCityM</t>
   </si>
   <si>
+    <t>assertEquals("must not be blank", driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[4]/div[1]/span[2]")) .getText());</t>
+  </si>
+  <si>
     <t>TestAddOwnerWithEmptyFirstName</t>
   </si>
   <si>
     <t>TestAddOwnerWithEmptyFirstNameM</t>
   </si>
   <si>
+    <t>assertEquals("must not be blank", driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[1]/div[1]/span[2]")) .getText());</t>
+  </si>
+  <si>
     <t>TestAddOwnerWithEmptyLastName</t>
   </si>
   <si>
     <t>TestAddOwnerWithEmptyLastNameM</t>
   </si>
   <si>
+    <t>assertEquals("must not be blank", driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[2]/div[1]/span[2]")) .getText());</t>
+  </si>
+  <si>
     <t>TestAddOwnerWithEmptyTelephone</t>
   </si>
   <si>
     <t>TestAddOwnerWithEmptyTelephoneM</t>
   </si>
   <si>
+    <t>assertTrue( driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[5]/div[1]/span[2]")) .getText().contains("must not be blank"));</t>
+  </si>
+  <si>
     <t>TestAddOwnerWithLongTelephone</t>
   </si>
   <si>
     <t>TestAddOwnerWithLongTelephoneM</t>
   </si>
   <si>
+    <t>assertTrue( driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[5]/div[1]/span[2]")) .getText().contains("Telephone must be a 10-digit number"));</t>
+  </si>
+  <si>
     <t>TestAddOwnerWithNotNumericTelephone</t>
   </si>
   <si>
@@ -126,18 +144,27 @@
     <t>TestAddOwnerWithValidDataM</t>
   </si>
   <si>
+    <t>assertEquals(firstName + " " + lastName, driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/table[1]/tbody[1]/tr[1]/td[1]/b[1]")) .getText(), "FirstName and LastName could not saved correctly");</t>
+  </si>
+  <si>
     <t>TestEditOwnerEmptyField</t>
   </si>
   <si>
     <t>TestEditOwnerEmptyFieldM</t>
   </si>
   <si>
+    <t>assertEquals("must not be blank", driver.findElement(By.className("help-inline")).getText());</t>
+  </si>
+  <si>
     <t>TestEditOwnerWithLongTelephone</t>
   </si>
   <si>
     <t>TestEditOwnerWithLongTelephoneM</t>
   </si>
   <si>
+    <t>assertEquals("Telephone must be a 10-digit number", driver.findElement(By.className("help-inline")).getText());</t>
+  </si>
+  <si>
     <t>TestEditOwnerWithNotNumericTelephone</t>
   </si>
   <si>
@@ -150,40 +177,61 @@
     <t>TestEditOwnerWithValidDataM</t>
   </si>
   <si>
+    <t>assertEquals(firstName + " " + lastName, driver.findElement(By.xpath("html[1]/body[1]/div[1]/div[1]/table[1]/tbody[1]/tr[1]/td[1]/b[1]")) .getText());</t>
+  </si>
+  <si>
     <t>TestFindAllOwner</t>
   </si>
   <si>
     <t>TestFindAllOwnerM</t>
   </si>
   <si>
+    <t>assertTrue(true);</t>
+  </si>
+  <si>
     <t>TestFindExistingOwner</t>
   </si>
   <si>
     <t>TestFindExistingOwnerM</t>
   </si>
   <si>
+    <t>assertTrue(driver.findElement(By.xpath("/html[1]/body[1]/div[1]/div[1]/table[1]/tbody[1]/tr[1]/td[1]/b[1]")) .getText().contains(lastName));</t>
+  </si>
+  <si>
     <t>TestFindExistingOwnerFromAll</t>
   </si>
   <si>
     <t>TestFindExistingOwnerFromAllM</t>
   </si>
   <si>
+    <t>assertEquals(owner, driver.findElement(By.xpath("//b[contains(text(),'George Franklin')]")).getText());</t>
+  </si>
+  <si>
     <t>TestFindNotExistingOwner</t>
   </si>
   <si>
     <t>TestFindNotExistingOwnerM</t>
   </si>
   <si>
+    <t>assertEquals("has not been found", driver.findElement( By.xpath("html[1]/body[1]/div[1]/div[1]/form[1]/div[1]/div[1]/div[1]/span[1]/div[1]/p[1]")) .getText());</t>
+  </si>
+  <si>
     <t>TestPetToOwner</t>
   </si>
   <si>
     <t>TestPetToOwnerM</t>
   </si>
   <si>
+    <t>assertEquals(petName, driver.findElement(By.xpath("//dd[contains(text()," + "'" + petName + "')]")).getText(), "Wrong petname added!");</t>
+  </si>
+  <si>
     <t>TestPetToOwnerWithEmptyField</t>
   </si>
   <si>
     <t>TestPetToOwnerWithEmptyFieldM</t>
+  </si>
+  <si>
+    <t>assertEquals(2, driver.findElements(By.className("help-inline")).size());</t>
   </si>
   <si>
     <t>mantisbt</t>
@@ -317,12 +365,53 @@
   <si>
     <t>Syntax error, missing method, wrong locator</t>
   </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.findElement(By.cssSelector("[type='submit']")).isDisplayed());</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.getPageSource().contains(firstName + " " + lastName));</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.getPageSource().contains(firstName));</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.getPageSource().contains(lastName));</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.getPageSource().contains(owner));</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.getPageSource().contains("No owners found"));</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.getPageSource().contains(petName));</t>
+  </si>
+  <si>
+    <t>org.junit.jupiter.api.Assertions.assertTrue(driver.findElement(By.id("owners")).isDisplayed());</t>
+  </si>
+  <si>
+    <t>org.opentest4j.AssertionFailedError: 
+Expected :true
+Actual   :false</t>
+  </si>
+  <si>
+    <t>Checks another objective: summit button visible instead of validation/error of the content.</t>
+  </si>
+  <si>
+    <t>Same intent but weaker as it should check a specific target element/value</t>
+  </si>
+  <si>
+    <t>Checks the wrong value</t>
+  </si>
+  <si>
+    <t>Gold assertion is tautological; generated adds UI constraint and is largely redundant with preceding findElement(By.id("owners"))</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -343,8 +432,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -369,8 +472,18 @@
         <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -422,11 +535,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -465,12 +593,37 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="29">
@@ -488,8 +641,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -502,12 +655,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -526,8 +673,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -540,12 +687,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -564,8 +705,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -578,12 +719,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -619,8 +754,8 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -633,12 +768,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -657,8 +786,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -671,12 +800,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -695,8 +818,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -709,12 +832,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -733,8 +850,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -747,12 +864,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -797,8 +908,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="left" vertical="center"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -811,12 +922,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -835,8 +940,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -849,12 +954,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -873,8 +972,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -887,12 +986,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -911,8 +1004,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -925,12 +1018,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -947,8 +1034,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <border>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -961,12 +1048,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -993,7 +1074,7 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1047,8 +1128,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L6" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25" totalsRowBorderDxfId="24">
-  <autoFilter ref="A1:L6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L55" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25" totalsRowBorderDxfId="24">
+  <autoFilter ref="A1:L55" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="App" totalsRowLabel="Total" dataDxfId="23" totalsRowDxfId="22"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Test Class" dataDxfId="21" totalsRowDxfId="20"/>
@@ -1361,7 +1442,7 @@
     <col min="4" max="4" width="31.28515625" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
     <col min="9" max="9" width="10.28515625" customWidth="1"/>
     <col min="10" max="10" width="40" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
@@ -1422,13 +1503,25 @@
       <c r="E2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15"/>
+      <c r="F2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H2" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
+      <c r="K2" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -1441,15 +1534,17 @@
         <v>14</v>
       </c>
       <c r="D3" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
-      <c r="I3" s="15"/>
+      <c r="I3" s="14"/>
       <c r="J3" s="12"/>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
@@ -1464,856 +1559,1048 @@
       <c r="C4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>18</v>
+      <c r="D4" s="12" t="s">
+        <v>19</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="12"/>
+      <c r="F4" s="12" t="s">
+        <v>17</v>
+      </c>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
-      <c r="I4" s="15"/>
+      <c r="I4" s="14"/>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
       <c r="L4" s="12"/>
     </row>
-    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H5" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-    </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>19</v>
-      </c>
       <c r="C6" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>18</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="12"/>
+      <c r="F6" s="12" t="s">
+        <v>22</v>
+      </c>
       <c r="G6" s="12"/>
       <c r="H6" s="12"/>
-      <c r="I6" s="15"/>
+      <c r="I6" s="14"/>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
       <c r="L6" s="12"/>
     </row>
-    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="12" t="s">
+    <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+    </row>
+    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-    </row>
-    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-    </row>
-    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-    </row>
-    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="E9" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+    </row>
+    <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>25</v>
+      </c>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
-      <c r="I10" s="15"/>
+      <c r="I10" s="17"/>
       <c r="J10" s="12"/>
       <c r="K10" s="12"/>
       <c r="L10" s="12"/>
     </row>
-    <row r="11" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="2" t="s">
+    <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-    </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="E11" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="H11" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="12"/>
+        <v>27</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>28</v>
+      </c>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
-      <c r="I12" s="15"/>
+      <c r="I12" s="17"/>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
       <c r="L12" s="12"/>
     </row>
-    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="12"/>
+        <v>27</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>28</v>
+      </c>
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
-      <c r="I13" s="15"/>
+      <c r="I13" s="17"/>
       <c r="J13" s="12"/>
       <c r="K13" s="12"/>
       <c r="L13" s="12"/>
     </row>
-    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="15"/>
+      <c r="E14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H14" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-    </row>
-    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K14" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L14" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
-      <c r="I15" s="15"/>
+      <c r="I15" s="17"/>
       <c r="J15" s="12"/>
       <c r="K15" s="12"/>
       <c r="L15" s="12"/>
     </row>
-    <row r="16" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
-      <c r="I16" s="15"/>
+      <c r="I16" s="17"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
       <c r="L16" s="12"/>
     </row>
-    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="15"/>
+      <c r="E17" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-    </row>
-    <row r="18" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K17" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L17" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" s="12"/>
+        <v>33</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
-      <c r="I18" s="15"/>
+      <c r="I18" s="17"/>
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
     </row>
-    <row r="19" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="12"/>
+        <v>33</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
-      <c r="I19" s="15"/>
+      <c r="I19" s="17"/>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
       <c r="L19" s="12"/>
     </row>
-    <row r="20" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="15"/>
+      <c r="E20" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H20" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
-    </row>
-    <row r="21" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K20" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L20" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F21" s="12"/>
+        <v>36</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
-      <c r="I21" s="15"/>
+      <c r="I21" s="17"/>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
     </row>
-    <row r="22" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F22" s="12"/>
+        <v>36</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
-      <c r="I22" s="15"/>
+      <c r="I22" s="17"/>
       <c r="J22" s="12"/>
       <c r="K22" s="12"/>
       <c r="L22" s="12"/>
     </row>
-    <row r="23" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="15"/>
+      <c r="E23" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="H23" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="12"/>
-    </row>
-    <row r="24" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K23" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L23" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F24" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
-      <c r="I24" s="15"/>
+      <c r="I24" s="17"/>
       <c r="J24" s="12"/>
       <c r="K24" s="12"/>
       <c r="L24" s="12"/>
     </row>
-    <row r="25" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F25" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>39</v>
+      </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
-      <c r="I25" s="15"/>
+      <c r="I25" s="17"/>
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
       <c r="L25" s="12"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="15"/>
+      <c r="E26" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K26" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L26" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F27" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
-      <c r="I27" s="15"/>
+      <c r="I27" s="17"/>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F28" s="12"/>
+        <v>41</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>42</v>
+      </c>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
-      <c r="I28" s="15"/>
+      <c r="I28" s="17"/>
       <c r="J28" s="12"/>
       <c r="K28" s="12"/>
       <c r="L28" s="12"/>
     </row>
-    <row r="29" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="15"/>
+      <c r="E29" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H29" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="12"/>
-    </row>
-    <row r="30" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K29" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L29" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
-      <c r="I30" s="15"/>
+      <c r="I30" s="17"/>
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
       <c r="L30" s="12"/>
     </row>
-    <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F31" s="12"/>
+        <v>44</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="G31" s="12"/>
       <c r="H31" s="12"/>
-      <c r="I31" s="15"/>
+      <c r="I31" s="17"/>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
       <c r="L31" s="12"/>
     </row>
-    <row r="32" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D32" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="15"/>
+      <c r="E32" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G32" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H32" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
-      <c r="L32" s="12"/>
-    </row>
-    <row r="33" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K32" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L32" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F33" s="12"/>
+        <v>47</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
-      <c r="I33" s="15"/>
+      <c r="I33" s="17"/>
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
       <c r="L33" s="12"/>
     </row>
-    <row r="34" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F34" s="12"/>
+        <v>47</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="G34" s="12"/>
       <c r="H34" s="12"/>
-      <c r="I34" s="15"/>
+      <c r="I34" s="17"/>
       <c r="J34" s="12"/>
       <c r="K34" s="12"/>
       <c r="L34" s="12"/>
     </row>
-    <row r="35" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
-      <c r="I35" s="15"/>
+      <c r="E35" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="H35" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
-      <c r="L35" s="12"/>
-    </row>
-    <row r="36" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K35" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L35" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F36" s="12"/>
+        <v>49</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>50</v>
+      </c>
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
-      <c r="I36" s="15"/>
+      <c r="I36" s="17"/>
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
       <c r="L36" s="12"/>
     </row>
-    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F37" s="12"/>
+        <v>49</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>50</v>
+      </c>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
-      <c r="I37" s="15"/>
+      <c r="I37" s="17"/>
       <c r="J37" s="12"/>
       <c r="K37" s="12"/>
       <c r="L37" s="12"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D38" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D38" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E38" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="15"/>
+      <c r="E38" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="H38" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
-      <c r="L38" s="12"/>
+      <c r="K38" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="L38" s="12" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F39" s="12"/>
+        <v>52</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E39" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>53</v>
+      </c>
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
-      <c r="I39" s="15"/>
+      <c r="I39" s="17"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
       <c r="L39" s="12"/>
@@ -2323,388 +2610,472 @@
         <v>12</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F40" s="12"/>
+        <v>52</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>53</v>
+      </c>
       <c r="G40" s="12"/>
       <c r="H40" s="12"/>
-      <c r="I40" s="15"/>
+      <c r="I40" s="17"/>
       <c r="J40" s="12"/>
       <c r="K40" s="12"/>
       <c r="L40" s="12"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D41" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E41" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F41" s="12"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="15"/>
+      <c r="E41" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F41" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="H41" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I41" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
-      <c r="L41" s="12"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K41" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L41" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E42" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F42" s="12"/>
+        <v>55</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>56</v>
+      </c>
       <c r="G42" s="12"/>
       <c r="H42" s="12"/>
-      <c r="I42" s="15"/>
+      <c r="I42" s="17"/>
       <c r="J42" s="12"/>
       <c r="K42" s="12"/>
       <c r="L42" s="12"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F43" s="12"/>
+        <v>55</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E43" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>56</v>
+      </c>
       <c r="G43" s="12"/>
       <c r="H43" s="12"/>
-      <c r="I43" s="15"/>
+      <c r="I43" s="17"/>
       <c r="J43" s="12"/>
       <c r="K43" s="12"/>
       <c r="L43" s="12"/>
     </row>
-    <row r="44" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D44" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D44" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E44" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="12"/>
-      <c r="I44" s="15"/>
+      <c r="E44" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G44" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H44" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I44" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
-      <c r="L44" s="12"/>
-    </row>
-    <row r="45" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K44" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L44" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F45" s="12"/>
+        <v>58</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>59</v>
+      </c>
       <c r="G45" s="12"/>
       <c r="H45" s="12"/>
-      <c r="I45" s="15"/>
+      <c r="I45" s="17"/>
       <c r="J45" s="12"/>
       <c r="K45" s="12"/>
       <c r="L45" s="12"/>
     </row>
-    <row r="46" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E46" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F46" s="12"/>
+        <v>58</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>59</v>
+      </c>
       <c r="G46" s="12"/>
       <c r="H46" s="12"/>
-      <c r="I46" s="15"/>
+      <c r="I46" s="17"/>
       <c r="J46" s="12"/>
       <c r="K46" s="12"/>
       <c r="L46" s="12"/>
     </row>
-    <row r="47" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D47" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E47" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-      <c r="L47" s="12"/>
-    </row>
-    <row r="48" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="E47" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G47" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="H47" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I47" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="J47" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="K47" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L47" s="12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E48" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F48" s="12"/>
+        <v>61</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E48" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>62</v>
+      </c>
       <c r="G48" s="12"/>
       <c r="H48" s="12"/>
-      <c r="I48" s="15"/>
+      <c r="I48" s="17"/>
       <c r="J48" s="12"/>
       <c r="K48" s="12"/>
       <c r="L48" s="12"/>
     </row>
-    <row r="49" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F49" s="12"/>
+        <v>61</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E49" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>62</v>
+      </c>
       <c r="G49" s="12"/>
       <c r="H49" s="12"/>
-      <c r="I49" s="15"/>
+      <c r="I49" s="17"/>
       <c r="J49" s="12"/>
       <c r="K49" s="12"/>
       <c r="L49" s="12"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D50" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E50" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F50" s="12"/>
-      <c r="G50" s="12"/>
-      <c r="H50" s="12"/>
-      <c r="I50" s="15"/>
+      <c r="E50" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="H50" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I50" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J50" s="12"/>
-      <c r="K50" s="12"/>
-      <c r="L50" s="12"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K50" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L50" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E51" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F51" s="12"/>
+        <v>64</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E51" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>65</v>
+      </c>
       <c r="G51" s="12"/>
       <c r="H51" s="12"/>
-      <c r="I51" s="15"/>
+      <c r="I51" s="17"/>
       <c r="J51" s="12"/>
       <c r="K51" s="12"/>
       <c r="L51" s="12"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F52" s="12"/>
+        <v>64</v>
+      </c>
+      <c r="D52" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F52" s="12" t="s">
+        <v>65</v>
+      </c>
       <c r="G52" s="12"/>
       <c r="H52" s="12"/>
-      <c r="I52" s="15"/>
+      <c r="I52" s="17"/>
       <c r="J52" s="12"/>
       <c r="K52" s="12"/>
       <c r="L52" s="12"/>
     </row>
-    <row r="53" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D53" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D53" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E53" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F53" s="12"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="12"/>
-      <c r="I53" s="15"/>
+      <c r="E53" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F53" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G53" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H53" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I53" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J53" s="12"/>
-      <c r="K53" s="12"/>
-      <c r="L53" s="12"/>
-    </row>
-    <row r="54" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="K53" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L53" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E54" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F54" s="12"/>
+        <v>67</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E54" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" s="12" t="s">
+        <v>68</v>
+      </c>
       <c r="G54" s="12"/>
       <c r="H54" s="12"/>
-      <c r="I54" s="15"/>
+      <c r="I54" s="17"/>
       <c r="J54" s="12"/>
       <c r="K54" s="12"/>
       <c r="L54" s="12"/>
     </row>
-    <row r="55" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C55" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E55" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F55" s="12"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="12"/>
-      <c r="I55" s="15"/>
-      <c r="J55" s="12"/>
-      <c r="K55" s="12"/>
-      <c r="L55" s="12"/>
+    <row r="55" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D55" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F55" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="18"/>
+      <c r="K55" s="18"/>
+      <c r="L55" s="18"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid classification" error="Please select a valid classification" promptTitle="Manual Classification" prompt="Select classification" sqref="K2:K6" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid classification" error="Please select a valid classification" promptTitle="Manual Classification" prompt="Select classification" sqref="K2:K55" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"correct,over_assertive,under_assertive,wrong_assertion,not_executable"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2773,243 +3144,243 @@
     </row>
     <row r="2" spans="1:12" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="H2" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="H4" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="H5" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="H6" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="H7" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="H8" s="2" t="b">
         <v>1</v>
       </c>
       <c r="I8" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="L8" s="2"/>
     </row>
@@ -3039,68 +3410,68 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
record results in the excel file
</commit_message>
<xml_diff>
--- a/Excel file summary.xlsx
+++ b/Excel file summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mezaj\projects\fstt_assignment\maven_selenium_project_Petclinic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF97F064-0C6B-4497-946B-C64C51C47F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159E7BE3-15A6-4752-8BDE-337BF54925A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="615" windowWidth="19395" windowHeight="20355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="149">
   <si>
     <t>App</t>
   </si>
@@ -405,6 +405,84 @@
   </si>
   <si>
     <t>Gold assertion is tautological; generated adds UI constraint and is largely redundant with preceding findElement(By.id("owners"))</t>
+  </si>
+  <si>
+    <t>assertTrue(driver.findElement(By.className("help-inline")).getText().contains("must not be blank"));</t>
+  </si>
+  <si>
+    <t>assertTrue(driver.findElement(By.className("help-inline")).getText().contains("Telephone must be a 10-digit number"));</t>
+  </si>
+  <si>
+    <t>assertEquals(firstName + " " + lastName, driver.findElement(By.xpath("//th[text()='Name']/following-sibling::td")).getText());</t>
+  </si>
+  <si>
+    <t>assertEquals(firstName + " " + lastName, driver.findElement(By.cssSelector("table.table-striped td b")).getText());</t>
+  </si>
+  <si>
+    <t>assertTrue(driver.findElement(By.id("owners")).isDisplayed());</t>
+  </si>
+  <si>
+    <t>assertTrue(driver.findElement(By.cssSelector("td b")).getText().contains(lastName));</t>
+  </si>
+  <si>
+    <t>assertEquals(owner, driver.findElement(By.cssSelector("table.table-striped td b")).getText());</t>
+  </si>
+  <si>
+    <t>assertEquals("has not been found", driver.findElement(By.className("help-inline")).getText());</t>
+  </si>
+  <si>
+    <t>assertEquals(petName, driver.findElement(By.xpath("//ddtext()='" + petName + "'")).getText());</t>
+  </si>
+  <si>
+    <t>Unable to locate element: {"method":"xpath","selector":"//button[text()='Add Pet']"}</t>
+  </si>
+  <si>
+    <t>Gold is trivial; generated adds stricter UI presence check.</t>
+  </si>
+  <si>
+    <t>Checks same expected validation text, locators differ</t>
+  </si>
+  <si>
+    <t>Same assertion intent and value, different selector.</t>
+  </si>
+  <si>
+    <t>Equivalent first-name empty-field error checks.</t>
+  </si>
+  <si>
+    <t>Empty last-name empty-field error checks.</t>
+  </si>
+  <si>
+    <t>Same telephone empty-field message check using contains.</t>
+  </si>
+  <si>
+    <t>Same telephone format error text check.</t>
+  </si>
+  <si>
+    <t>Same non-numeric telephone error message check.</t>
+  </si>
+  <si>
+    <t>Same owner full-name equality check after save; alternate locator.</t>
+  </si>
+  <si>
+    <t>Exact same assertion semantics as gold.</t>
+  </si>
+  <si>
+    <t>Same edited owner full-name equality check; different locator style.</t>
+  </si>
+  <si>
+    <t>Same logic: result contains searched last name</t>
+  </si>
+  <si>
+    <t>Ads extra structural constraint beyond gold intent.</t>
+  </si>
+  <si>
+    <t>Same "has not been found" message check; different locator.</t>
+  </si>
+  <si>
+    <t>Generated assertion/locator is invalid or not runnable in context.</t>
+  </si>
+  <si>
+    <t>Exact same check: two validation errors expected.</t>
   </si>
 </sst>
 </file>
@@ -554,7 +632,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -602,16 +680,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
@@ -1431,6 +1506,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="651" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{F01F5FA2-2A42-46A3-A35D-47871AED28D1}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;e314c4cd-7aa9-4dfe-9e2e-4946fa76416f&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L55"/>
@@ -1568,12 +1665,22 @@
       <c r="F4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="14"/>
+      <c r="G4" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
+      <c r="K4" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
@@ -1638,30 +1745,40 @@
       <c r="L6" s="12"/>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="18" t="s">
+      <c r="A7" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="18" t="s">
+      <c r="E7" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
+      <c r="G7" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="L7" s="17" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -1700,30 +1817,30 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="18" t="s">
+      <c r="A9" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
     </row>
     <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
@@ -1744,43 +1861,53 @@
       <c r="F10" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="17"/>
+      <c r="G10" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H10" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
+      <c r="K10" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="18" t="s">
+      <c r="A11" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="18" t="s">
+      <c r="E11" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="G11" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="H11" s="18" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18" t="s">
+      <c r="H11" s="17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17" t="s">
         <v>77</v>
       </c>
       <c r="L11" s="12" t="s">
@@ -1808,7 +1935,7 @@
       </c>
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
-      <c r="I12" s="17"/>
+      <c r="I12" s="14"/>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
       <c r="L12" s="12"/>
@@ -1832,12 +1959,22 @@
       <c r="F13" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="17"/>
+      <c r="G13" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
+      <c r="K13" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L13" s="12" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
@@ -1896,7 +2033,7 @@
       </c>
       <c r="G15" s="12"/>
       <c r="H15" s="12"/>
-      <c r="I15" s="17"/>
+      <c r="I15" s="14"/>
       <c r="J15" s="12"/>
       <c r="K15" s="12"/>
       <c r="L15" s="12"/>
@@ -1920,12 +2057,22 @@
       <c r="F16" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="17"/>
+      <c r="G16" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="H16" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="12"/>
+      <c r="K16" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L16" s="12" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="17" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
@@ -1984,7 +2131,7 @@
       </c>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
-      <c r="I18" s="17"/>
+      <c r="I18" s="14"/>
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
@@ -2008,12 +2155,22 @@
       <c r="F19" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="17"/>
+      <c r="G19" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="H19" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
+      <c r="K19" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L19" s="12" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="20" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
@@ -2072,7 +2229,7 @@
       </c>
       <c r="G21" s="12"/>
       <c r="H21" s="12"/>
-      <c r="I21" s="17"/>
+      <c r="I21" s="14"/>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
@@ -2096,12 +2253,22 @@
       <c r="F22" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="17"/>
+      <c r="G22" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="H22" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
+      <c r="K22" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L22" s="12" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="23" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
@@ -2160,7 +2327,7 @@
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
-      <c r="I24" s="17"/>
+      <c r="I24" s="14"/>
       <c r="J24" s="12"/>
       <c r="K24" s="12"/>
       <c r="L24" s="12"/>
@@ -2184,12 +2351,22 @@
       <c r="F25" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="17"/>
+      <c r="G25" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="H25" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
+      <c r="K25" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L25" s="12" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="26" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
@@ -2248,7 +2425,7 @@
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
-      <c r="I27" s="17"/>
+      <c r="I27" s="14"/>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
@@ -2272,12 +2449,22 @@
       <c r="F28" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="17"/>
+      <c r="G28" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H28" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="12"/>
+      <c r="K28" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="29" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
@@ -2336,7 +2523,7 @@
       </c>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
-      <c r="I30" s="17"/>
+      <c r="I30" s="14"/>
       <c r="J30" s="12"/>
       <c r="K30" s="12"/>
       <c r="L30" s="12"/>
@@ -2360,12 +2547,22 @@
       <c r="F31" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="17"/>
+      <c r="G31" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H31" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-      <c r="L31" s="12"/>
+      <c r="K31" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L31" s="12" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="32" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
@@ -2424,7 +2621,7 @@
       </c>
       <c r="G33" s="12"/>
       <c r="H33" s="12"/>
-      <c r="I33" s="17"/>
+      <c r="I33" s="14"/>
       <c r="J33" s="12"/>
       <c r="K33" s="12"/>
       <c r="L33" s="12"/>
@@ -2448,12 +2645,22 @@
       <c r="F34" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="17"/>
+      <c r="G34" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H34" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I34" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
+      <c r="K34" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L34" s="12" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="35" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
@@ -2512,7 +2719,7 @@
       </c>
       <c r="G36" s="12"/>
       <c r="H36" s="12"/>
-      <c r="I36" s="17"/>
+      <c r="I36" s="14"/>
       <c r="J36" s="12"/>
       <c r="K36" s="12"/>
       <c r="L36" s="12"/>
@@ -2536,12 +2743,22 @@
       <c r="F37" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="17"/>
+      <c r="G37" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="H37" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
-      <c r="L37" s="12"/>
+      <c r="K37" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L37" s="12" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="38" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
@@ -2600,12 +2817,12 @@
       </c>
       <c r="G39" s="12"/>
       <c r="H39" s="12"/>
-      <c r="I39" s="17"/>
+      <c r="I39" s="14"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12"/>
       <c r="L39" s="12"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
         <v>12</v>
       </c>
@@ -2624,12 +2841,22 @@
       <c r="F40" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="17"/>
+      <c r="G40" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="H40" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
-      <c r="L40" s="12"/>
+      <c r="K40" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="L40" s="12" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
@@ -2688,7 +2915,7 @@
       </c>
       <c r="G42" s="12"/>
       <c r="H42" s="12"/>
-      <c r="I42" s="17"/>
+      <c r="I42" s="14"/>
       <c r="J42" s="12"/>
       <c r="K42" s="12"/>
       <c r="L42" s="12"/>
@@ -2712,12 +2939,22 @@
       <c r="F43" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="17"/>
+      <c r="G43" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="H43" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
-      <c r="L43" s="12"/>
+      <c r="K43" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L43" s="12" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="44" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
@@ -2776,7 +3013,7 @@
       </c>
       <c r="G45" s="12"/>
       <c r="H45" s="12"/>
-      <c r="I45" s="17"/>
+      <c r="I45" s="14"/>
       <c r="J45" s="12"/>
       <c r="K45" s="12"/>
       <c r="L45" s="12"/>
@@ -2800,12 +3037,22 @@
       <c r="F46" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="G46" s="12"/>
-      <c r="H46" s="12"/>
-      <c r="I46" s="17"/>
+      <c r="G46" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="H46" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I46" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-      <c r="L46" s="12"/>
+      <c r="K46" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="L46" s="12" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="47" spans="1:12" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
@@ -2832,7 +3079,7 @@
       <c r="H47" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="I47" s="22" t="s">
+      <c r="I47" s="21" t="s">
         <v>93</v>
       </c>
       <c r="J47" s="12" t="s">
@@ -2866,7 +3113,7 @@
       </c>
       <c r="G48" s="12"/>
       <c r="H48" s="12"/>
-      <c r="I48" s="17"/>
+      <c r="I48" s="14"/>
       <c r="J48" s="12"/>
       <c r="K48" s="12"/>
       <c r="L48" s="12"/>
@@ -2890,12 +3137,22 @@
       <c r="F49" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="G49" s="12"/>
-      <c r="H49" s="12"/>
-      <c r="I49" s="17"/>
+      <c r="G49" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H49" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I49" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="J49" s="12"/>
-      <c r="K49" s="12"/>
-      <c r="L49" s="12"/>
+      <c r="K49" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="L49" s="12" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="50" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
@@ -2954,7 +3211,7 @@
       </c>
       <c r="G51" s="12"/>
       <c r="H51" s="12"/>
-      <c r="I51" s="17"/>
+      <c r="I51" s="14"/>
       <c r="J51" s="12"/>
       <c r="K51" s="12"/>
       <c r="L51" s="12"/>
@@ -2978,12 +3235,24 @@
       <c r="F52" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="G52" s="12"/>
-      <c r="H52" s="12"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="12"/>
-      <c r="K52" s="12"/>
-      <c r="L52" s="12"/>
+      <c r="G52" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="H52" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I52" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="J52" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="K52" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="L52" s="12" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="53" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
@@ -3042,36 +3311,46 @@
       </c>
       <c r="G54" s="12"/>
       <c r="H54" s="12"/>
-      <c r="I54" s="17"/>
+      <c r="I54" s="14"/>
       <c r="J54" s="12"/>
       <c r="K54" s="12"/>
       <c r="L54" s="12"/>
     </row>
     <row r="55" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" s="18" t="s">
+      <c r="A55" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="C55" s="18" t="s">
+      <c r="C55" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="D55" s="18" t="s">
+      <c r="D55" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="E55" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F55" s="18" t="s">
+      <c r="E55" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F55" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="18"/>
-      <c r="K55" s="18"/>
-      <c r="L55" s="18"/>
+      <c r="G55" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="H55" s="17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I55" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="J55" s="17"/>
+      <c r="K55" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="L55" s="17" t="s">
+        <v>148</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>